<commit_message>
loaded targets and market prices
</commit_message>
<xml_diff>
--- a/data_files/DAILY PRICE REPORT 22-05-2026.xlsx
+++ b/data_files/DAILY PRICE REPORT 22-05-2026.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dashboard-inventory\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBAA69F4-0477-494C-BAD8-556BC51E9E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{330812CA-AAFE-43F0-BF9F-67610E6BF2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="87">
   <si>
     <t>PRODUCT</t>
   </si>
@@ -124,12 +123,6 @@
     <t>MIX XYLENE - HAZIRA</t>
   </si>
   <si>
-    <t>MIX-ISOMER - KANDLA</t>
-  </si>
-  <si>
-    <t>ISOMER -MIX XYLENE  -PIPAVAV</t>
-  </si>
-  <si>
     <t>ORTHO - HAZIRA</t>
   </si>
   <si>
@@ -262,9 +255,6 @@
     <t xml:space="preserve">METHANOL - KAKINADA </t>
   </si>
   <si>
-    <t>MIX HEPTANE-KANDLA</t>
-  </si>
-  <si>
     <t>2 ETHYL HEXANOL -KANDLA</t>
   </si>
   <si>
@@ -295,107 +285,23 @@
     <t>NEXT WEEK ARRIVAL</t>
   </si>
   <si>
-    <t>2-ETHYLHEXANOL</t>
-  </si>
-  <si>
-    <t>ACETIC ACID</t>
-  </si>
-  <si>
-    <t>BUTYL ACETATE</t>
-  </si>
-  <si>
-    <t>BUTYL DI  GLYCOL</t>
-  </si>
-  <si>
-    <t>BUTYL GLYCOL</t>
-  </si>
-  <si>
-    <t>C-9</t>
-  </si>
-  <si>
-    <t>CYCLOHEXANE</t>
-  </si>
-  <si>
-    <t>CYCLOHEXANONE</t>
-  </si>
-  <si>
-    <t>DEG</t>
-  </si>
-  <si>
-    <t>EDC</t>
-  </si>
-  <si>
-    <t>HEXANE</t>
-  </si>
-  <si>
-    <t>IBA</t>
-  </si>
-  <si>
-    <t>IPA</t>
-  </si>
-  <si>
-    <t>MEG</t>
-  </si>
-  <si>
-    <t>METHANOL</t>
-  </si>
-  <si>
-    <t>MIX XYLENE</t>
-  </si>
-  <si>
-    <t>MIX XYLENE ISOMER GR</t>
-  </si>
-  <si>
-    <t>MIXED HEPTANE</t>
-  </si>
-  <si>
-    <t>MMA</t>
-  </si>
-  <si>
-    <t>N-PROPANOL</t>
-  </si>
-  <si>
-    <t>NORMAL BUTANOL</t>
-  </si>
-  <si>
-    <t>ORTHO XYLENE</t>
-  </si>
-  <si>
-    <t>PHENOL-M</t>
-  </si>
-  <si>
-    <t>POLYLOL 0434</t>
-  </si>
-  <si>
-    <t>POLYLOL 0656</t>
-  </si>
-  <si>
-    <t>POLYOL 1127</t>
-  </si>
-  <si>
-    <t>PROPIONIC ACID</t>
-  </si>
-  <si>
-    <t>PROPYLENE GLYCOL</t>
-  </si>
-  <si>
-    <t>STYRENE MONOMER</t>
-  </si>
-  <si>
-    <t>NAMES IN PRICING SHEET</t>
-  </si>
-  <si>
-    <t>Mapped Names from Inventory Sheet</t>
-  </si>
-  <si>
-    <t>Unmapped Names from Inventory Sheet</t>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>MIX HEPTANE - KANDLA</t>
+  </si>
+  <si>
+    <t>MIX ISOMER - KANDLA</t>
+  </si>
+  <si>
+    <t>MIX ISOMER  -PIPAVAV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,22 +322,8 @@
       <name val="Arial Black"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -450,26 +342,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="15">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -609,59 +483,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -741,12 +567,6 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -765,21 +585,6 @@
     <xf numFmtId="1" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1060,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T63"/>
+  <dimension ref="A1:T62"/>
   <sheetFormatPr defaultColWidth="21" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.5546875" customWidth="1"/>
@@ -1162,7 +967,7 @@
         <f t="shared" ref="H2:H24" si="0">G2-D2</f>
         <v>2702.3530000000001</v>
       </c>
-      <c r="I2" s="33">
+      <c r="I2" s="31">
         <v>35284</v>
       </c>
       <c r="J2" s="8">
@@ -1170,7 +975,7 @@
         <v>1119</v>
       </c>
       <c r="K2" s="9">
-        <f t="shared" ref="K2:K23" si="2">(J2*M$61+2500)/1000</f>
+        <f t="shared" ref="K2:K23" si="2">(J2*M$62+2500)/1000</f>
         <v>111.32275</v>
       </c>
       <c r="L2" s="9">
@@ -1211,7 +1016,7 @@
         <f t="shared" si="0"/>
         <v>603.22700000000077</v>
       </c>
-      <c r="I3" s="34"/>
+      <c r="I3" s="32"/>
       <c r="J3" s="8">
         <f t="shared" si="1"/>
         <v>1119</v>
@@ -1234,7 +1039,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="10"/>
       <c r="S3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="T3">
         <v>1019</v>
@@ -1283,7 +1088,7 @@
       <c r="P4" s="5"/>
       <c r="Q4" s="10"/>
       <c r="S4" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T4">
         <v>1049</v>
@@ -1333,7 +1138,7 @@
       <c r="P5" s="12"/>
       <c r="Q5" s="10"/>
       <c r="S5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="T5">
         <v>1031</v>
@@ -1382,7 +1187,7 @@
       <c r="P6" s="5"/>
       <c r="Q6" s="10"/>
       <c r="S6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="T6">
         <v>1059</v>
@@ -1432,7 +1237,7 @@
       <c r="P7" s="5"/>
       <c r="Q7" s="10"/>
       <c r="S7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="T7">
         <v>1264</v>
@@ -1463,7 +1268,7 @@
         <f t="shared" si="0"/>
         <v>-645.18599999999992</v>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="28">
         <v>30030</v>
       </c>
       <c r="J8" s="8">
@@ -1490,7 +1295,7 @@
         <v>20</v>
       </c>
       <c r="S8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="T8">
         <v>915</v>
@@ -1517,7 +1322,7 @@
         <f t="shared" si="0"/>
         <v>844.66000000000099</v>
       </c>
-      <c r="I9" s="31"/>
+      <c r="I9" s="29"/>
       <c r="J9" s="8">
         <f t="shared" si="1"/>
         <v>1131</v>
@@ -1631,7 +1436,7 @@
     </row>
     <row r="12" spans="1:20" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>21</v>
@@ -1651,7 +1456,7 @@
         <f t="shared" si="0"/>
         <v>306.45400000000001</v>
       </c>
-      <c r="I12" s="30"/>
+      <c r="I12" s="28"/>
       <c r="J12" s="8">
         <f t="shared" si="1"/>
         <v>1149</v>
@@ -1678,7 +1483,7 @@
     </row>
     <row r="13" spans="1:20" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>26</v>
@@ -1694,7 +1499,7 @@
         <f t="shared" si="0"/>
         <v>1973.616</v>
       </c>
-      <c r="I13" s="32"/>
+      <c r="I13" s="30"/>
       <c r="J13" s="8">
         <f t="shared" si="1"/>
         <v>1149</v>
@@ -1721,7 +1526,7 @@
     </row>
     <row r="14" spans="1:20" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>18</v>
@@ -1737,7 +1542,7 @@
         <f t="shared" si="0"/>
         <v>1517.2829999999999</v>
       </c>
-      <c r="I14" s="31"/>
+      <c r="I14" s="29"/>
       <c r="J14" s="8">
         <f t="shared" si="1"/>
         <v>1149</v>
@@ -1761,7 +1566,7 @@
     </row>
     <row r="15" spans="1:20" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>18</v>
@@ -1806,7 +1611,7 @@
     </row>
     <row r="16" spans="1:20" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>18</v>
@@ -1850,7 +1655,7 @@
     </row>
     <row r="17" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>18</v>
@@ -1892,7 +1697,7 @@
     </row>
     <row r="18" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>21</v>
@@ -1910,7 +1715,7 @@
         <f t="shared" si="0"/>
         <v>2621.4169999999999</v>
       </c>
-      <c r="I18" s="30">
+      <c r="I18" s="28">
         <v>26471</v>
       </c>
       <c r="J18" s="8">
@@ -1937,7 +1742,7 @@
     </row>
     <row r="19" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>18</v>
@@ -1960,7 +1765,7 @@
         <f t="shared" si="0"/>
         <v>-2311.556</v>
       </c>
-      <c r="I19" s="31"/>
+      <c r="I19" s="29"/>
       <c r="J19" s="8">
         <f>L19+295</f>
         <v>1210</v>
@@ -1991,7 +1796,7 @@
     </row>
     <row r="20" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>21</v>
@@ -2012,7 +1817,7 @@
         <f t="shared" si="0"/>
         <v>751.8449999999998</v>
       </c>
-      <c r="I20" s="32"/>
+      <c r="I20" s="30"/>
       <c r="J20" s="8">
         <v>1800</v>
       </c>
@@ -2035,7 +1840,7 @@
     </row>
     <row r="21" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>18</v>
@@ -2056,7 +1861,7 @@
         <f t="shared" si="0"/>
         <v>514.03600000000006</v>
       </c>
-      <c r="I21" s="31"/>
+      <c r="I21" s="29"/>
       <c r="J21" s="8">
         <v>1800</v>
       </c>
@@ -2084,7 +1889,7 @@
     </row>
     <row r="22" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>18</v>
@@ -2126,7 +1931,7 @@
     </row>
     <row r="23" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>21</v>
@@ -2164,10 +1969,10 @@
     </row>
     <row r="24" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="7">
@@ -2182,12 +1987,12 @@
         <f t="shared" si="0"/>
         <v>328.22199999999998</v>
       </c>
-      <c r="I24" s="31"/>
+      <c r="I24" s="29"/>
       <c r="J24" s="8">
         <v>2000</v>
       </c>
       <c r="K24" s="9">
-        <f>(J24*M$61*1.0825+2500)/1000</f>
+        <f>(J24*M$62*1.0825+2500)/1000</f>
         <v>213.04624999999999</v>
       </c>
       <c r="L24" s="9" t="s">
@@ -2201,12 +2006,12 @@
         <v>235</v>
       </c>
       <c r="Q24" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>26</v>
@@ -2223,14 +2028,14 @@
       <c r="H25" s="7">
         <v>0</v>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="28">
         <v>13425</v>
       </c>
       <c r="J25" s="8">
         <v>1420</v>
       </c>
       <c r="K25" s="9">
-        <f>(J25*M$61*1.0275+2500)/1000</f>
+        <f>(J25*M$62*1.0275+2500)/1000</f>
         <v>144.39261250000001</v>
       </c>
       <c r="L25" s="9">
@@ -2247,7 +2052,7 @@
     </row>
     <row r="26" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>18</v>
@@ -2273,7 +2078,7 @@
         <v>1670</v>
       </c>
       <c r="K26" s="9">
-        <f>(J26*M$61*1.0825+2500)/1000</f>
+        <f>(J26*M$62*1.0825+2500)/1000</f>
         <v>178.30611875</v>
       </c>
       <c r="L26" s="9" t="s">
@@ -2290,12 +2095,12 @@
         <v>160</v>
       </c>
       <c r="Q26" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>18</v>
@@ -2322,7 +2127,7 @@
         <v>707.5</v>
       </c>
       <c r="K27" s="9">
-        <f>(J27*M$61+2500)/1000</f>
+        <f>(J27*M$62+2500)/1000</f>
         <v>71.304374999999993</v>
       </c>
       <c r="L27" s="9">
@@ -2340,7 +2145,7 @@
     </row>
     <row r="28" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>26</v>
@@ -2369,7 +2174,7 @@
         <v>815</v>
       </c>
       <c r="K28" s="9">
-        <f>(J28*M$61*1.0825+2500)/1000</f>
+        <f>(J28*M$62*1.0825+2500)/1000</f>
         <v>88.297596874999996</v>
       </c>
       <c r="L28" s="9">
@@ -2384,12 +2189,12 @@
         <v>84</v>
       </c>
       <c r="Q28" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>26</v>
@@ -2418,7 +2223,7 @@
         <v>450</v>
       </c>
       <c r="K29" s="9">
-        <f>(J29*M$61+1500)/1000</f>
+        <f>(J29*M$62+1500)/1000</f>
         <v>45.262500000000003</v>
       </c>
       <c r="L29" s="8">
@@ -2436,7 +2241,7 @@
     </row>
     <row r="30" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>18</v>
@@ -2462,7 +2267,7 @@
         <v>450</v>
       </c>
       <c r="K30" s="9">
-        <f>(J30*M$61+1500)/1000</f>
+        <f>(J30*M$62+1500)/1000</f>
         <v>45.262500000000003</v>
       </c>
       <c r="L30" s="8">
@@ -2480,7 +2285,7 @@
     </row>
     <row r="31" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>18</v>
@@ -2505,7 +2310,7 @@
         <v>1885</v>
       </c>
       <c r="K31" s="9">
-        <f>(J31*M$61*1.0825+2500)/1000</f>
+        <f>(J31*M$62*1.0825+2500)/1000</f>
         <v>200.93984062500002</v>
       </c>
       <c r="L31" s="8">
@@ -2521,7 +2326,7 @@
     </row>
     <row r="32" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>18</v>
@@ -2547,7 +2352,7 @@
         <v>1000</v>
       </c>
       <c r="K32" s="9">
-        <f>(J32*M$61*1.0825+2500)/1000</f>
+        <f>(J32*M$62*1.0825+2500)/1000</f>
         <v>107.77312499999999</v>
       </c>
       <c r="L32" s="9" t="s">
@@ -2565,7 +2370,7 @@
     </row>
     <row r="33" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>21</v>
@@ -2589,7 +2394,7 @@
         <v>1000</v>
       </c>
       <c r="K33" s="9">
-        <f>(J33*M$61*1.0825+2500)/1000</f>
+        <f>(J33*M$62*1.0825+2500)/1000</f>
         <v>107.77312499999999</v>
       </c>
       <c r="L33" s="9" t="s">
@@ -2609,7 +2414,7 @@
     </row>
     <row r="34" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>18</v>
@@ -2639,7 +2444,7 @@
         <v>1450</v>
       </c>
       <c r="K34" s="9">
-        <f>(J34*M$61*1.0825+2500)/1000</f>
+        <f>(J34*M$62*1.0825+2500)/1000</f>
         <v>155.14603124999999</v>
       </c>
       <c r="L34" s="9" t="s">
@@ -2654,12 +2459,12 @@
       </c>
       <c r="P34" s="5"/>
       <c r="Q34" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>18</v>
@@ -2686,7 +2491,7 @@
         <v>1500</v>
       </c>
       <c r="K35" s="9">
-        <f>(J35*M$61*1.055+2500)/1000</f>
+        <f>(J35*M$62*1.055+2500)/1000</f>
         <v>156.39812499999999</v>
       </c>
       <c r="L35" s="9"/>
@@ -2700,10 +2505,10 @@
     </row>
     <row r="36" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C36" s="5">
         <v>1000</v>
@@ -2718,14 +2523,14 @@
         <f t="shared" si="3"/>
         <v>763.46799999999985</v>
       </c>
-      <c r="I36" s="30">
+      <c r="I36" s="28">
         <v>5309</v>
       </c>
       <c r="J36" s="8">
         <v>1100</v>
       </c>
       <c r="K36" s="9">
-        <f>(J36*M$61*1.0825+2500)/1000</f>
+        <f>(J36*M$62*1.0825+2500)/1000</f>
         <v>118.3004375</v>
       </c>
       <c r="L36" s="9" t="s">
@@ -2747,7 +2552,7 @@
     </row>
     <row r="37" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>26</v>
@@ -2771,7 +2576,7 @@
         <v>1350</v>
       </c>
       <c r="K37" s="9">
-        <f>(J37*M$61*1.0825+2500)/1000</f>
+        <f>(J37*M$62*1.0825+2500)/1000</f>
         <v>144.61871875</v>
       </c>
       <c r="L37" s="9" t="s">
@@ -2787,7 +2592,7 @@
     </row>
     <row r="38" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>26</v>
@@ -2815,7 +2620,7 @@
         <v>1350</v>
       </c>
       <c r="K38" s="9">
-        <f>(J38*M$61*1.0825+2500)/1000</f>
+        <f>(J38*M$62*1.0825+2500)/1000</f>
         <v>144.61871875</v>
       </c>
       <c r="L38" s="9" t="s">
@@ -2833,7 +2638,7 @@
     </row>
     <row r="39" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>18</v>
@@ -2858,7 +2663,7 @@
         <v>1200</v>
       </c>
       <c r="K39" s="9">
-        <f>(J39*M$61*1.0825+2500)/1000</f>
+        <f>(J39*M$62*1.0825+2500)/1000</f>
         <v>128.82775000000001</v>
       </c>
       <c r="L39" s="9" t="s">
@@ -2874,7 +2679,7 @@
     </row>
     <row r="40" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>18</v>
@@ -2905,7 +2710,7 @@
         <v>1330</v>
       </c>
       <c r="K40" s="9">
-        <f>(J40*M$61+2500)/1000</f>
+        <f>(J40*M$62+2500)/1000</f>
         <v>131.8425</v>
       </c>
       <c r="L40" s="9">
@@ -2921,12 +2726,12 @@
       </c>
       <c r="P40" s="5"/>
       <c r="Q40" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>18</v>
@@ -2952,7 +2757,7 @@
         <v>350</v>
       </c>
       <c r="K41" s="9">
-        <f>(J41*M$61+2500)/1000</f>
+        <f>(J41*M$62+2500)/1000</f>
         <v>36.537500000000001</v>
       </c>
       <c r="L41" s="9"/>
@@ -2968,7 +2773,7 @@
     </row>
     <row r="42" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>18</v>
@@ -2995,7 +2800,7 @@
         <v>1300</v>
       </c>
       <c r="K42" s="9">
-        <f>(J42*M$61*1.0825+2500)/1000</f>
+        <f>(J42*M$62*1.0825+2500)/1000</f>
         <v>139.3550625</v>
       </c>
       <c r="L42" s="5"/>
@@ -3009,10 +2814,10 @@
     </row>
     <row r="43" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C43" s="5">
         <v>1500</v>
@@ -3034,7 +2839,7 @@
         <v>1250</v>
       </c>
       <c r="K43" s="9">
-        <f t="shared" ref="K43:K52" si="5">(J43*M$61+2500)/1000</f>
+        <f t="shared" ref="K43:K52" si="5">(J43*M$62+2500)/1000</f>
         <v>124.0625</v>
       </c>
       <c r="L43" s="9">
@@ -3050,7 +2855,7 @@
     </row>
     <row r="44" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>18</v>
@@ -3071,7 +2876,7 @@
         <f t="shared" si="4"/>
         <v>1315.66</v>
       </c>
-      <c r="I44" s="30">
+      <c r="I44" s="28">
         <v>543</v>
       </c>
       <c r="J44" s="9">
@@ -3095,7 +2900,7 @@
     </row>
     <row r="45" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>26</v>
@@ -3117,7 +2922,7 @@
         <f t="shared" si="4"/>
         <v>17.599999999999902</v>
       </c>
-      <c r="I45" s="31"/>
+      <c r="I45" s="29"/>
       <c r="J45" s="9">
         <v>1250</v>
       </c>
@@ -3137,12 +2942,12 @@
       </c>
       <c r="P45" s="5"/>
       <c r="Q45" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>18</v>
@@ -3186,7 +2991,7 @@
     </row>
     <row r="47" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>21</v>
@@ -3227,7 +3032,7 @@
     </row>
     <row r="48" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>18</v>
@@ -3251,7 +3056,7 @@
         <f t="shared" si="4"/>
         <v>39.3599999999999</v>
       </c>
-      <c r="I48" s="30">
+      <c r="I48" s="28">
         <v>5601</v>
       </c>
       <c r="J48" s="9">
@@ -3280,10 +3085,10 @@
     </row>
     <row r="49" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="7">
@@ -3298,7 +3103,7 @@
         <f t="shared" si="4"/>
         <v>684.36099999999988</v>
       </c>
-      <c r="I49" s="32"/>
+      <c r="I49" s="30"/>
       <c r="J49" s="9">
         <v>1170</v>
       </c>
@@ -3322,10 +3127,10 @@
     </row>
     <row r="50" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="7"/>
@@ -3338,7 +3143,7 @@
         <f t="shared" si="4"/>
         <v>151</v>
       </c>
-      <c r="I50" s="31"/>
+      <c r="I50" s="29"/>
       <c r="J50" s="9">
         <v>1170</v>
       </c>
@@ -3362,7 +3167,7 @@
     </row>
     <row r="51" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>21</v>
@@ -3407,7 +3212,7 @@
     </row>
     <row r="52" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>18</v>
@@ -3452,7 +3257,7 @@
     </row>
     <row r="53" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B53" s="12" t="s">
         <v>18</v>
@@ -3478,7 +3283,7 @@
         <v>1150</v>
       </c>
       <c r="K53" s="9">
-        <f>(J53*M$61*1.0825+2500)/1000</f>
+        <f>(J53*M$62*1.0825+2500)/1000</f>
         <v>123.56409375</v>
       </c>
       <c r="L53" s="9">
@@ -3496,7 +3301,7 @@
     </row>
     <row r="54" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A54" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B54" s="12" t="s">
         <v>18</v>
@@ -3523,7 +3328,7 @@
         <v>1150</v>
       </c>
       <c r="K54" s="9">
-        <f>(J54*M$61*1.0825+2500)/1000</f>
+        <f>(J54*M$62*1.0825+2500)/1000</f>
         <v>123.56409375</v>
       </c>
       <c r="L54" s="9">
@@ -3542,7 +3347,7 @@
     </row>
     <row r="55" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>18</v>
@@ -3571,7 +3376,7 @@
         <v>605</v>
       </c>
       <c r="K55" s="9">
-        <f>(J55*M$61*1.0275+1500)/1000</f>
+        <f>(J55*M$62*1.0275+1500)/1000</f>
         <v>61.954246875000003</v>
       </c>
       <c r="L55" s="9">
@@ -3593,7 +3398,7 @@
     </row>
     <row r="56" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A56" s="12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>18</v>
@@ -3619,7 +3424,7 @@
         <v>605</v>
       </c>
       <c r="K56" s="9">
-        <f>(J56*M$61*1.0275+1800)/1000</f>
+        <f>(J56*M$62*1.0275+1800)/1000</f>
         <v>62.254246875000007</v>
       </c>
       <c r="L56" s="9">
@@ -3637,7 +3442,7 @@
     </row>
     <row r="57" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A57" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B57" s="12" t="s">
         <v>18</v>
@@ -3668,7 +3473,7 @@
         <v>605</v>
       </c>
       <c r="K57" s="9">
-        <f>(J57*M$61*1.0275+1500)/1000</f>
+        <f>(J57*M$62*1.0275+1500)/1000</f>
         <v>61.954246875000003</v>
       </c>
       <c r="L57" s="9">
@@ -3685,12 +3490,12 @@
       </c>
       <c r="P57" s="5"/>
       <c r="Q57" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="58" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A58" s="12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B58" s="12" t="s">
         <v>18</v>
@@ -3720,7 +3525,7 @@
         <v>605</v>
       </c>
       <c r="K58" s="9">
-        <f>(J58*M$61*1.0275+2000)/1000</f>
+        <f>(J58*M$62*1.0275+2000)/1000</f>
         <v>62.454246875000003</v>
       </c>
       <c r="L58" s="9">
@@ -3742,7 +3547,7 @@
     </row>
     <row r="59" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="B59" s="12" t="s">
         <v>18</v>
@@ -3771,7 +3576,7 @@
         <v>1005</v>
       </c>
       <c r="K59" s="9">
-        <f>(J59*M$61*1.0275+2500)/1000</f>
+        <f>(J59*M$62*1.0275+2500)/1000</f>
         <v>102.92399687500001</v>
       </c>
       <c r="L59" s="9">
@@ -3788,9 +3593,9 @@
       <c r="P59" s="5"/>
       <c r="Q59" s="9"/>
     </row>
-    <row r="60" spans="1:17" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B60" s="12" t="s">
         <v>18</v>
@@ -3800,8 +3605,8 @@
         <f>875-20-30-21-25</f>
         <v>779</v>
       </c>
-      <c r="E60" s="33"/>
-      <c r="F60" s="33"/>
+      <c r="E60" s="31"/>
+      <c r="F60" s="31"/>
       <c r="G60" s="7">
         <f>33.41+475</f>
         <v>508.40999999999997</v>
@@ -3817,7 +3622,7 @@
         <v>1250</v>
       </c>
       <c r="K60" s="9">
-        <f>(J60*M$61*1.0825+2500)/1000</f>
+        <f>(J60*M$62*1.0825+2500)/1000</f>
         <v>134.09140625000001</v>
       </c>
       <c r="L60" s="10">
@@ -3836,527 +3641,91 @@
       <c r="Q60" s="10"/>
     </row>
     <row r="61" spans="1:17" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="29"/>
-      <c r="B61" s="22"/>
-      <c r="C61" s="23">
-        <f t="shared" ref="C61:I61" si="6">SUM(C2:C60)</f>
+      <c r="A61" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B61" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C61" s="14"/>
+      <c r="D61" s="6">
+        <f>139.02-25</f>
+        <v>114.02000000000001</v>
+      </c>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="7">
+        <f>D61</f>
+        <v>114.02000000000001</v>
+      </c>
+      <c r="H61" s="6">
+        <f>G61-D61</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="11">
+        <v>33273</v>
+      </c>
+      <c r="J61" s="8">
+        <v>540</v>
+      </c>
+      <c r="K61" s="9">
+        <f>(J61*M$62+2500)/1000</f>
+        <v>55.015000000000001</v>
+      </c>
+      <c r="L61" s="9"/>
+      <c r="M61" s="5"/>
+      <c r="N61" s="5">
+        <v>40</v>
+      </c>
+      <c r="O61" s="12"/>
+      <c r="P61" s="12"/>
+      <c r="Q61" s="10"/>
+    </row>
+    <row r="62" spans="1:17" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="B62" s="22"/>
+      <c r="C62" s="23">
+        <f t="shared" ref="C62:I62" si="6">SUM(C2:C60)</f>
         <v>85660</v>
       </c>
-      <c r="D61" s="6">
+      <c r="D62" s="6">
         <f t="shared" si="6"/>
         <v>29038.872570000007</v>
       </c>
-      <c r="E61" s="6">
+      <c r="E62" s="6">
         <f t="shared" si="6"/>
         <v>30045.864999999998</v>
       </c>
-      <c r="F61" s="6">
+      <c r="F62" s="6">
         <f t="shared" si="6"/>
         <v>4775</v>
       </c>
-      <c r="G61" s="24">
+      <c r="G62" s="24">
         <f t="shared" si="6"/>
         <v>78047.984570000001</v>
       </c>
-      <c r="H61" s="25">
+      <c r="H62" s="25">
         <f t="shared" si="6"/>
         <v>49778.915000000008</v>
       </c>
-      <c r="I61" s="26">
+      <c r="I62" s="26">
         <f t="shared" si="6"/>
         <v>203805</v>
       </c>
-      <c r="J61" s="8"/>
-      <c r="K61" s="5"/>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5">
+      <c r="J62" s="8"/>
+      <c r="K62" s="5"/>
+      <c r="L62" s="5"/>
+      <c r="M62" s="5">
         <v>97.25</v>
       </c>
-      <c r="N61" s="5"/>
-      <c r="O61" s="5"/>
-      <c r="P61" s="5"/>
-      <c r="Q61" s="10"/>
-    </row>
-    <row r="62" spans="1:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="A62" s="14"/>
-      <c r="B62" s="27"/>
-      <c r="C62" s="14"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="28"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14"/>
-      <c r="K62" s="14"/>
-      <c r="L62" s="14"/>
-      <c r="M62" s="14"/>
-      <c r="N62" s="14"/>
-      <c r="O62" s="14"/>
-      <c r="P62" s="14"/>
-      <c r="Q62" s="14"/>
-    </row>
-    <row r="63" spans="1:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B63" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="C63" s="14"/>
-      <c r="D63" s="6">
-        <f>139.02-25</f>
-        <v>114.02000000000001</v>
-      </c>
-      <c r="E63" s="6"/>
-      <c r="F63" s="6"/>
-      <c r="G63" s="7" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H63" s="6" t="e">
-        <f>G63-D63</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I63" s="11">
-        <v>33273</v>
-      </c>
-      <c r="J63" s="8">
-        <v>540</v>
-      </c>
-      <c r="K63" s="9">
-        <f>(J63*M$61+2500)/1000</f>
-        <v>55.015000000000001</v>
-      </c>
-      <c r="L63" s="9"/>
-      <c r="M63" s="5"/>
-      <c r="N63" s="5">
-        <v>40</v>
-      </c>
-      <c r="O63" s="12"/>
-      <c r="P63" s="12"/>
-      <c r="Q63" s="10"/>
+      <c r="N62" s="5"/>
+      <c r="O62" s="5"/>
+      <c r="P62" s="5"/>
+      <c r="Q62" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFE916C5-E693-41D3-B71E-B267520939F9}">
-  <dimension ref="A1:C60"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="26.5546875" style="45" customWidth="1"/>
-    <col min="2" max="2" width="40.5546875" style="43" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" style="44" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="38"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="35" t="s">
-        <v>115</v>
-      </c>
-      <c r="B1" s="36" t="s">
-        <v>116</v>
-      </c>
-      <c r="C1" s="37" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="B2" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="41"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="42" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="42" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="43" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="B6" s="43" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="42" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="42" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="42" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="42" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="43" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="42" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="42" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="42" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="42" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="C16" s="44" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="42" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="44" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="42" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="42" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="43" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="42" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="43" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="B21" s="43" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="42" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="43" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="42" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="43" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="42" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="42" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="42" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="42" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" s="43" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="42" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="42" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="42" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="42" t="s">
-        <v>75</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="B35" s="43" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="42" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="42" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="42" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="43" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="42" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="42" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="42" t="s">
-        <v>45</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="42" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="43" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="42" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="42" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="42" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="42" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="42" t="s">
-        <v>50</v>
-      </c>
-      <c r="B48" s="43" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="42" t="s">
-        <v>31</v>
-      </c>
-      <c r="B49" s="43" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="42" t="s">
-        <v>58</v>
-      </c>
-      <c r="B51" s="43" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="42" t="s">
-        <v>49</v>
-      </c>
-      <c r="B52" s="43" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C53" s="44" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="42" t="s">
-        <v>84</v>
-      </c>
-      <c r="B54" s="43" t="s">
-        <v>114</v>
-      </c>
-      <c r="C54" s="44" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="B55" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="44" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="C56" s="44" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="42" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="42" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="42" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="42" t="s">
-        <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A60">
-    <sortCondition ref="A2:A60"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>